<commit_message>
Final analysis and text
</commit_message>
<xml_diff>
--- a/Material/2. Interviews & Surveys/Attribute Definition.xlsx
+++ b/Material/2. Interviews & Surveys/Attribute Definition.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\franc\Documents\GitHub\DSE_thesis\Material\2. Interviews &amp; Surveys\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2015489-4BD5-411D-9955-359D0D2AFBE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{903896E5-AFB6-4679-AD4A-63AC3B88E702}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="824" activeTab="3" xr2:uid="{1010D4BD-99A2-4997-AD21-2857331DB82F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="824" activeTab="2" xr2:uid="{1010D4BD-99A2-4997-AD21-2857331DB82F}"/>
   </bookViews>
   <sheets>
     <sheet name="Improvement" sheetId="9" r:id="rId1"/>
@@ -1608,7 +1608,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1715,9 +1715,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1726,6 +1723,18 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="34" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -2137,68 +2146,68 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="37" t="s">
+      <c r="A2" s="36" t="s">
         <v>181</v>
       </c>
-      <c r="C2" s="37" t="s">
+      <c r="C2" s="36" t="s">
         <v>102</v>
       </c>
-      <c r="E2" s="37" t="s">
+      <c r="E2" s="36" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="37" t="s">
+      <c r="A3" s="36" t="s">
         <v>182</v>
       </c>
-      <c r="C3" s="37" t="s">
+      <c r="C3" s="36" t="s">
         <v>103</v>
       </c>
-      <c r="E3" s="37" t="s">
+      <c r="E3" s="36" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="36" t="s">
         <v>183</v>
       </c>
-      <c r="C4" s="37" t="s">
+      <c r="C4" s="36" t="s">
         <v>104</v>
       </c>
-      <c r="E4" s="37" t="s">
+      <c r="E4" s="36" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="37" t="s">
+      <c r="A5" s="36" t="s">
         <v>184</v>
       </c>
-      <c r="C5" s="37" t="s">
+      <c r="C5" s="36" t="s">
         <v>105</v>
       </c>
-      <c r="E5" s="37" t="s">
+      <c r="E5" s="36" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="36" t="s">
         <v>185</v>
       </c>
-      <c r="C6" s="37" t="s">
+      <c r="C6" s="36" t="s">
         <v>106</v>
       </c>
-      <c r="E6" s="37" t="s">
+      <c r="E6" s="36" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="37" t="s">
+      <c r="A7" s="36" t="s">
         <v>186</v>
       </c>
-      <c r="C7" s="37" t="s">
+      <c r="C7" s="36" t="s">
         <v>142</v>
       </c>
-      <c r="E7" s="37" t="s">
+      <c r="E7" s="36" t="s">
         <v>285</v>
       </c>
       <c r="F7" s="25" t="s">
@@ -2206,41 +2215,41 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="37" t="s">
+      <c r="A8" s="36" t="s">
         <v>187</v>
       </c>
-      <c r="C8" s="37" t="s">
+      <c r="C8" s="36" t="s">
         <v>143</v>
       </c>
-      <c r="E8" s="37" t="s">
+      <c r="E8" s="36" t="s">
         <v>170</v>
       </c>
       <c r="F8" s="13"/>
     </row>
     <row r="9" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="37" t="s">
+      <c r="A9" s="36" t="s">
         <v>188</v>
       </c>
-      <c r="C9" s="37" t="s">
+      <c r="C9" s="36" t="s">
         <v>58</v>
       </c>
-      <c r="E9" s="38" t="s">
+      <c r="E9" s="37" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C10" s="37" t="s">
+      <c r="C10" s="36" t="s">
         <v>132</v>
       </c>
-      <c r="E10" s="37" t="s">
+      <c r="E10" s="36" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C11" s="37" t="s">
+      <c r="C11" s="36" t="s">
         <v>144</v>
       </c>
-      <c r="E11" s="37" t="s">
+      <c r="E11" s="36" t="s">
         <v>174</v>
       </c>
       <c r="F11" s="13"/>
@@ -4348,15 +4357,15 @@
   <dimension ref="A1:B24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="63.77734375" style="7" customWidth="1"/>
-    <col min="2" max="2" width="116.21875" customWidth="1"/>
+    <col min="1" max="1" width="63" style="7" customWidth="1"/>
+    <col min="2" max="2" width="63" style="42" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="19" t="s">
+      <c r="A1" s="39" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="41" t="s">
         <v>222</v>
       </c>
     </row>
@@ -4364,7 +4373,7 @@
       <c r="A2" s="11" t="s">
         <v>145</v>
       </c>
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="40" t="s">
         <v>239</v>
       </c>
     </row>
@@ -4372,7 +4381,7 @@
       <c r="A3" s="11" t="s">
         <v>146</v>
       </c>
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="40" t="s">
         <v>239</v>
       </c>
     </row>
@@ -4380,7 +4389,7 @@
       <c r="A4" s="11" t="s">
         <v>147</v>
       </c>
-      <c r="B4" s="29" t="s">
+      <c r="B4" s="40" t="s">
         <v>239</v>
       </c>
     </row>
@@ -4388,7 +4397,7 @@
       <c r="A5" s="11" t="s">
         <v>148</v>
       </c>
-      <c r="B5" s="29" t="s">
+      <c r="B5" s="40" t="s">
         <v>239</v>
       </c>
     </row>
@@ -4396,7 +4405,7 @@
       <c r="A6" s="11" t="s">
         <v>149</v>
       </c>
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="40" t="s">
         <v>239</v>
       </c>
     </row>
@@ -4404,7 +4413,7 @@
       <c r="A7" s="11" t="s">
         <v>150</v>
       </c>
-      <c r="B7" s="29" t="s">
+      <c r="B7" s="40" t="s">
         <v>239</v>
       </c>
     </row>
@@ -4412,15 +4421,15 @@
       <c r="A8" s="11" t="s">
         <v>151</v>
       </c>
-      <c r="B8" s="29" t="s">
+      <c r="B8" s="40" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>152</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="40" t="s">
         <v>268</v>
       </c>
     </row>
@@ -4428,7 +4437,7 @@
       <c r="A10" s="11" t="s">
         <v>153</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="40" t="s">
         <v>269</v>
       </c>
     </row>
@@ -4436,7 +4445,7 @@
       <c r="A11" s="11" t="s">
         <v>154</v>
       </c>
-      <c r="B11" s="29" t="s">
+      <c r="B11" s="40" t="s">
         <v>270</v>
       </c>
     </row>
@@ -4444,15 +4453,15 @@
       <c r="A12" s="11" t="s">
         <v>155</v>
       </c>
-      <c r="B12" s="29" t="s">
+      <c r="B12" s="40" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
         <v>156</v>
       </c>
-      <c r="B13" s="36" t="s">
+      <c r="B13" s="40" t="s">
         <v>271</v>
       </c>
     </row>
@@ -4460,7 +4469,7 @@
       <c r="A14" s="11" t="s">
         <v>157</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="40" t="s">
         <v>272</v>
       </c>
     </row>
@@ -4468,7 +4477,7 @@
       <c r="A15" s="11" t="s">
         <v>158</v>
       </c>
-      <c r="B15" s="29" t="s">
+      <c r="B15" s="40" t="s">
         <v>273</v>
       </c>
     </row>
@@ -4476,7 +4485,7 @@
       <c r="A16" s="11" t="s">
         <v>159</v>
       </c>
-      <c r="B16" s="29" t="s">
+      <c r="B16" s="40" t="s">
         <v>274</v>
       </c>
     </row>
@@ -4484,7 +4493,7 @@
       <c r="A17" s="11" t="s">
         <v>160</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="40" t="s">
         <v>276</v>
       </c>
     </row>
@@ -4492,7 +4501,7 @@
       <c r="A18" s="11" t="s">
         <v>161</v>
       </c>
-      <c r="B18" s="29" t="s">
+      <c r="B18" s="40" t="s">
         <v>239</v>
       </c>
     </row>
@@ -4500,7 +4509,7 @@
       <c r="A19" s="11" t="s">
         <v>162</v>
       </c>
-      <c r="B19" s="29" t="s">
+      <c r="B19" s="40" t="s">
         <v>239</v>
       </c>
     </row>
@@ -4508,7 +4517,7 @@
       <c r="A20" s="11" t="s">
         <v>163</v>
       </c>
-      <c r="B20" s="29" t="s">
+      <c r="B20" s="40" t="s">
         <v>239</v>
       </c>
     </row>
@@ -4516,7 +4525,7 @@
       <c r="A21" s="11" t="s">
         <v>164</v>
       </c>
-      <c r="B21" s="29" t="s">
+      <c r="B21" s="40" t="s">
         <v>239</v>
       </c>
     </row>
@@ -4524,7 +4533,7 @@
       <c r="A22" s="11" t="s">
         <v>165</v>
       </c>
-      <c r="B22" s="29" t="s">
+      <c r="B22" s="40" t="s">
         <v>239</v>
       </c>
     </row>
@@ -4532,15 +4541,15 @@
       <c r="A23" s="11" t="s">
         <v>166</v>
       </c>
-      <c r="B23" s="29" t="s">
+      <c r="B23" s="40" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="11" t="s">
         <v>167</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="40" t="s">
         <v>275</v>
       </c>
     </row>
@@ -4747,10 +4756,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="39" t="s">
+      <c r="A1" s="38" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="38" t="s">
         <v>222</v>
       </c>
     </row>
@@ -4762,7 +4771,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>288</v>
       </c>
@@ -4770,7 +4779,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>290</v>
       </c>
@@ -4835,7 +4844,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="38" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="10"/>

</xml_diff>